<commit_message>
Add GitHub tasks for Mutoni to the task sheet
</commit_message>
<xml_diff>
--- a/BSE_Group_Assignments_Task_Sheet_PCA_Formative2_Team15.xlsx
+++ b/BSE_Group_Assignments_Task_Sheet_PCA_Formative2_Team15.xlsx
@@ -396,7 +396,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1006"/>
+  <dimension ref="A1:Y1009"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="21.13" customWidth="1" style="12" min="1" max="1"/>
@@ -1050,7 +1050,7 @@
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Run the notebook in Google Colab and verify every output</t>
+          <t>Run the notebook in Google Colab, verify every output, and post a short verification note on GitHub (an Issue or a comment)</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -1093,16 +1093,16 @@
       <c r="X17" s="2" t="n"/>
       <c r="Y17" s="2" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" s="12">
       <c r="A18" s="9" t="n"/>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Combine notebook PDF and task sheet PDF, final check, submit</t>
+          <t>GitHub: accept the collaborator invite, work on a branch and open a pull request for Nelly to review</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Teta Butera Nelly and Mutoni Keira</t>
+          <t>Mutoni Keira</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1120,11 +1120,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Repo created; combined PDF to be rebuilt after the written answers are added.</t>
-        </is>
-      </c>
+      <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
@@ -1144,117 +1140,105 @@
       <c r="X18" s="2" t="n"/>
       <c r="Y18" s="2" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" s="12">
       <c r="A19" s="9" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="2" t="n"/>
-      <c r="R19" s="2" t="n"/>
-      <c r="S19" s="2" t="n"/>
-      <c r="T19" s="2" t="n"/>
-      <c r="U19" s="2" t="n"/>
-      <c r="V19" s="2" t="n"/>
-      <c r="W19" s="2" t="n"/>
-      <c r="X19" s="2" t="n"/>
-      <c r="Y19" s="2" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Meeting Attendance Log</t>
+          <t>GitHub: add a "How to run in Colab" section and a results summary to the README (own words)</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="n"/>
-      <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="n"/>
-      <c r="W20" s="2" t="n"/>
-      <c r="X20" s="2" t="n"/>
-      <c r="Y20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Meeting Date</t>
+          <t>Mutoni Keira</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Agenda</t>
+          <t>2026-09-30</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Facilitator</t>
+          <t>Not started</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Attendees</t>
+          <t>No</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="G19" s="13" t="inlineStr"/>
+    </row>
+    <row r="20" s="12">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Key Discussion Points</t>
+          <t>GitHub: write data/DATA_DICTIONARY.md describing the 15 features and the added sub_region column</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Next Steps</t>
+          <t>Mutoni Keira</t>
         </is>
       </c>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="n"/>
-      <c r="T21" s="2" t="n"/>
-      <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
-      <c r="W21" s="2" t="n"/>
-      <c r="X21" s="2" t="n"/>
-      <c r="Y21" s="2" t="n"/>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21" s="12">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Rebuild the combined PDF with the final answers, commit it to the repo, final check, submit</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Teta Butera Nelly and Mutoni Keira</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>Repo created; combined PDF to be rebuilt after the written answers are added.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
@@ -1275,13 +1259,11 @@
       <c r="Y22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="n"/>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Meeting Attendance Log</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
@@ -1302,13 +1284,37 @@
       <c r="Y23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
-      <c r="G24" s="9" t="n"/>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Meeting Date</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Facilitator</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Attendees</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Key Discussion Points</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Next Steps</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
@@ -1384,12 +1390,12 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
+      <c r="B27" s="9" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
@@ -1411,12 +1417,12 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
+      <c r="B28" s="9" t="n"/>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9" t="n"/>
+      <c r="F28" s="9" t="n"/>
+      <c r="G28" s="9" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
@@ -1438,12 +1444,12 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
@@ -1599,7 +1605,7 @@
       <c r="Y34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="n"/>
+      <c r="A35" s="9" t="n"/>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n"/>
@@ -1626,7 +1632,7 @@
       <c r="Y35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n"/>
+      <c r="A36" s="9" t="n"/>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
@@ -1653,7 +1659,7 @@
       <c r="Y36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n"/>
+      <c r="A37" s="9" t="n"/>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
@@ -1680,7 +1686,7 @@
       <c r="Y37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n"/>
+      <c r="A38" s="10" t="n"/>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
@@ -1707,7 +1713,7 @@
       <c r="Y38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
+      <c r="A39" s="11" t="n"/>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
@@ -1788,7 +1794,7 @@
       <c r="Y41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n"/>
+      <c r="A42" s="2" t="n"/>
       <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
@@ -1923,7 +1929,7 @@
       <c r="Y46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
+      <c r="A47" s="11" t="n"/>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
@@ -2004,7 +2010,7 @@
       <c r="Y49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n"/>
+      <c r="A50" s="2" t="n"/>
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
@@ -2139,7 +2145,7 @@
       <c r="Y54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
+      <c r="A55" s="11" t="n"/>
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
@@ -2220,7 +2226,7 @@
       <c r="Y57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="n"/>
+      <c r="A58" s="2" t="n"/>
       <c r="B58" s="2" t="n"/>
       <c r="C58" s="2" t="n"/>
       <c r="D58" s="2" t="n"/>
@@ -2355,7 +2361,7 @@
       <c r="Y62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
+      <c r="A63" s="11" t="n"/>
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n"/>
@@ -2382,7 +2388,7 @@
       <c r="Y63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
+      <c r="A64" s="11" t="n"/>
       <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="n"/>
       <c r="D64" s="2" t="n"/>
@@ -2409,7 +2415,7 @@
       <c r="Y64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
+      <c r="A65" s="11" t="n"/>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
@@ -27842,17 +27848,98 @@
       <c r="X1006" s="2" t="n"/>
       <c r="Y1006" s="2" t="n"/>
     </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="n"/>
+      <c r="B1007" s="2" t="n"/>
+      <c r="C1007" s="2" t="n"/>
+      <c r="D1007" s="2" t="n"/>
+      <c r="E1007" s="2" t="n"/>
+      <c r="F1007" s="2" t="n"/>
+      <c r="G1007" s="2" t="n"/>
+      <c r="H1007" s="2" t="n"/>
+      <c r="I1007" s="2" t="n"/>
+      <c r="J1007" s="2" t="n"/>
+      <c r="K1007" s="2" t="n"/>
+      <c r="L1007" s="2" t="n"/>
+      <c r="M1007" s="2" t="n"/>
+      <c r="N1007" s="2" t="n"/>
+      <c r="O1007" s="2" t="n"/>
+      <c r="P1007" s="2" t="n"/>
+      <c r="Q1007" s="2" t="n"/>
+      <c r="R1007" s="2" t="n"/>
+      <c r="S1007" s="2" t="n"/>
+      <c r="T1007" s="2" t="n"/>
+      <c r="U1007" s="2" t="n"/>
+      <c r="V1007" s="2" t="n"/>
+      <c r="W1007" s="2" t="n"/>
+      <c r="X1007" s="2" t="n"/>
+      <c r="Y1007" s="2" t="n"/>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="n"/>
+      <c r="B1008" s="2" t="n"/>
+      <c r="C1008" s="2" t="n"/>
+      <c r="D1008" s="2" t="n"/>
+      <c r="E1008" s="2" t="n"/>
+      <c r="F1008" s="2" t="n"/>
+      <c r="G1008" s="2" t="n"/>
+      <c r="H1008" s="2" t="n"/>
+      <c r="I1008" s="2" t="n"/>
+      <c r="J1008" s="2" t="n"/>
+      <c r="K1008" s="2" t="n"/>
+      <c r="L1008" s="2" t="n"/>
+      <c r="M1008" s="2" t="n"/>
+      <c r="N1008" s="2" t="n"/>
+      <c r="O1008" s="2" t="n"/>
+      <c r="P1008" s="2" t="n"/>
+      <c r="Q1008" s="2" t="n"/>
+      <c r="R1008" s="2" t="n"/>
+      <c r="S1008" s="2" t="n"/>
+      <c r="T1008" s="2" t="n"/>
+      <c r="U1008" s="2" t="n"/>
+      <c r="V1008" s="2" t="n"/>
+      <c r="W1008" s="2" t="n"/>
+      <c r="X1008" s="2" t="n"/>
+      <c r="Y1008" s="2" t="n"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="2" t="n"/>
+      <c r="B1009" s="2" t="n"/>
+      <c r="C1009" s="2" t="n"/>
+      <c r="D1009" s="2" t="n"/>
+      <c r="E1009" s="2" t="n"/>
+      <c r="F1009" s="2" t="n"/>
+      <c r="G1009" s="2" t="n"/>
+      <c r="H1009" s="2" t="n"/>
+      <c r="I1009" s="2" t="n"/>
+      <c r="J1009" s="2" t="n"/>
+      <c r="K1009" s="2" t="n"/>
+      <c r="L1009" s="2" t="n"/>
+      <c r="M1009" s="2" t="n"/>
+      <c r="N1009" s="2" t="n"/>
+      <c r="O1009" s="2" t="n"/>
+      <c r="P1009" s="2" t="n"/>
+      <c r="Q1009" s="2" t="n"/>
+      <c r="R1009" s="2" t="n"/>
+      <c r="S1009" s="2" t="n"/>
+      <c r="T1009" s="2" t="n"/>
+      <c r="U1009" s="2" t="n"/>
+      <c r="V1009" s="2" t="n"/>
+      <c r="W1009" s="2" t="n"/>
+      <c r="X1009" s="2" t="n"/>
+      <c r="Y1009" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E10:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E10:E21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Completed,Did not participate"</formula1>
     </dataValidation>
-    <dataValidation sqref="F10:F18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F10:F21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>